<commit_message>
Updated Attack Surface Analysis - Model Creation template (added additional port interfaces)
</commit_message>
<xml_diff>
--- a/distribution/reference_documents/templates/AVCDL attack surface analysis model template.xlsx
+++ b/distribution/reference_documents/templates/AVCDL attack surface analysis model template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10402"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10413"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charles.wilson/Documents/projects/AVCDL/source/reference_documents/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B765ED69-ABC5-8C43-9FE3-6D4EED4F6694}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16BFF26B-DA7D-0B4A-B05A-B9D102082DDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="41840" yWindow="940" windowWidth="30240" windowHeight="18880" xr2:uid="{DEA20EDE-F7A8-FC4F-9F8A-95A2B1030BD3}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="96">
   <si>
     <t>DO NOT EDIT THIS PAGE</t>
   </si>
@@ -172,12 +172,6 @@
   </si>
   <si>
     <t>JTAG</t>
-  </si>
-  <si>
-    <t>RS232</t>
-  </si>
-  <si>
-    <t>RS422</t>
   </si>
   <si>
     <t>USB</t>
@@ -338,6 +332,24 @@
   </si>
   <si>
     <t>Model Revision</t>
+  </si>
+  <si>
+    <t>serial</t>
+  </si>
+  <si>
+    <t>parallel</t>
+  </si>
+  <si>
+    <t>PS/2</t>
+  </si>
+  <si>
+    <t>video</t>
+  </si>
+  <si>
+    <t>audio</t>
+  </si>
+  <si>
+    <t>other</t>
   </si>
 </sst>
 </file>
@@ -906,7 +918,7 @@
   <sheetData>
     <row r="2" spans="2:11" ht="63" x14ac:dyDescent="0.75">
       <c r="B2" s="24" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C2" s="24"/>
       <c r="D2" s="24"/>
@@ -920,11 +932,11 @@
     </row>
     <row r="4" spans="2:11" ht="32" x14ac:dyDescent="0.4">
       <c r="B4" s="8" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C4" s="6"/>
       <c r="D4" s="26" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E4" s="26"/>
       <c r="F4" s="26"/>
@@ -935,11 +947,11 @@
     </row>
     <row r="6" spans="2:11" ht="32" x14ac:dyDescent="0.4">
       <c r="B6" s="8" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C6" s="6"/>
       <c r="D6" s="26" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E6" s="26"/>
       <c r="F6" s="26"/>
@@ -950,7 +962,7 @@
     </row>
     <row r="8" spans="2:11" ht="32" x14ac:dyDescent="0.4">
       <c r="B8" s="8" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C8" s="6"/>
       <c r="D8" s="26"/>
@@ -963,11 +975,11 @@
     </row>
     <row r="10" spans="2:11" ht="32" x14ac:dyDescent="0.4">
       <c r="B10" s="8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="27" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E10" s="27"/>
       <c r="F10" s="27"/>
@@ -978,11 +990,11 @@
     </row>
     <row r="12" spans="2:11" ht="32" x14ac:dyDescent="0.4">
       <c r="B12" s="8" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="27" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E12" s="27"/>
       <c r="F12" s="27"/>
@@ -993,11 +1005,11 @@
     </row>
     <row r="14" spans="2:11" ht="32" x14ac:dyDescent="0.4">
       <c r="B14" s="8" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="27" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E14" s="27"/>
       <c r="F14" s="27"/>
@@ -1008,7 +1020,7 @@
     </row>
     <row r="16" spans="2:11" ht="32" x14ac:dyDescent="0.4">
       <c r="B16" s="8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C16" s="6"/>
       <c r="D16" s="28">
@@ -1023,7 +1035,7 @@
     </row>
     <row r="18" spans="2:11" ht="32" x14ac:dyDescent="0.4">
       <c r="B18" s="8" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="9">
@@ -1037,7 +1049,7 @@
     </row>
     <row r="20" spans="2:11" ht="32" x14ac:dyDescent="0.4">
       <c r="B20" s="25" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C20" s="25"/>
       <c r="D20" s="25"/>
@@ -1093,7 +1105,7 @@
   <sheetData>
     <row r="2" spans="1:7" ht="63" x14ac:dyDescent="0.75">
       <c r="B2" s="29" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -1104,13 +1116,13 @@
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
       <c r="B4" s="12" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -1119,7 +1131,7 @@
       </c>
       <c r="C5" s="17"/>
       <c r="D5" s="19" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -1216,7 +1228,7 @@
   <sheetData>
     <row r="2" spans="1:7" ht="63" x14ac:dyDescent="0.75">
       <c r="B2" s="29" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -1227,13 +1239,13 @@
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
       <c r="B4" s="14" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -1331,7 +1343,7 @@
   <sheetData>
     <row r="2" spans="2:10" ht="63" x14ac:dyDescent="0.75">
       <c r="B2" s="29" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -1344,7 +1356,7 @@
     </row>
     <row r="5" spans="2:10" ht="27" x14ac:dyDescent="0.35">
       <c r="B5" s="30" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C5" s="30"/>
       <c r="D5" s="30"/>
@@ -1380,7 +1392,7 @@
   <sheetData>
     <row r="2" spans="1:12" ht="63" x14ac:dyDescent="0.75">
       <c r="B2" s="29" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -1411,10 +1423,10 @@
         <v>4</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
@@ -1569,9 +1581,9 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" showInputMessage="1" showErrorMessage="1" xr:uid="{DD42BC24-35AA-F347-B7EB-2DE43F25FBC5}">
+        <x14:dataValidation type="list" showInputMessage="1" showErrorMessage="1" xr:uid="{B22D7C0C-3E28-1449-A3A2-23C86C225061}">
           <x14:formula1>
-            <xm:f>legend!$A$2:$A$8</xm:f>
+            <xm:f>legend!$A$2:$A$12</xm:f>
           </x14:formula1>
           <xm:sqref>D5:D20</xm:sqref>
         </x14:dataValidation>
@@ -1595,7 +1607,7 @@
   <sheetData>
     <row r="2" spans="1:12" ht="63" x14ac:dyDescent="0.75">
       <c r="B2" s="29" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -1613,7 +1625,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>37</v>
@@ -1625,10 +1637,10 @@
         <v>4</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
@@ -1821,7 +1833,7 @@
   <sheetData>
     <row r="2" spans="1:12" ht="63" x14ac:dyDescent="0.75">
       <c r="B2" s="29" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -1843,10 +1855,10 @@
         <v>2</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>3</v>
@@ -1855,10 +1867,10 @@
         <v>4</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
@@ -2062,15 +2074,15 @@
         <v>38</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="21" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B2" s="22" t="s">
         <v>39</v>
@@ -2079,15 +2091,15 @@
         <v>40</v>
       </c>
       <c r="D2" s="21" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="21" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B3" s="22" t="s">
         <v>35</v>
@@ -2096,15 +2108,15 @@
         <v>5</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E3" s="21" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="21" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B4" s="22" t="s">
         <v>36</v>
@@ -2113,10 +2125,10 @@
         <v>6</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -2130,13 +2142,13 @@
         <v>8</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E5" s="21"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="21" t="s">
-        <v>43</v>
+        <v>90</v>
       </c>
       <c r="B6" s="22" t="s">
         <v>9</v>
@@ -2149,20 +2161,20 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="21" t="s">
-        <v>44</v>
+        <v>91</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D7" s="21"/>
       <c r="E7" s="21"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="21" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B8" s="22" t="s">
         <v>11</v>
@@ -2174,7 +2186,9 @@
       <c r="E8" s="21"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="21"/>
+      <c r="A9" s="21" t="s">
+        <v>92</v>
+      </c>
       <c r="B9" s="22" t="s">
         <v>13</v>
       </c>
@@ -2185,7 +2199,9 @@
       <c r="E9" s="21"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" s="21"/>
+      <c r="A10" s="21" t="s">
+        <v>93</v>
+      </c>
       <c r="B10" s="22" t="s">
         <v>15</v>
       </c>
@@ -2196,7 +2212,9 @@
       <c r="E10" s="21"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" s="21"/>
+      <c r="A11" s="21" t="s">
+        <v>94</v>
+      </c>
       <c r="B11" s="22" t="s">
         <v>17</v>
       </c>
@@ -2207,7 +2225,9 @@
       <c r="E11" s="21"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" s="21"/>
+      <c r="A12" s="21" t="s">
+        <v>95</v>
+      </c>
       <c r="B12" s="22" t="s">
         <v>19</v>
       </c>
@@ -2242,10 +2262,10 @@
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="21"/>
       <c r="B15" s="22" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C15" s="20" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D15" s="21"/>
       <c r="E15" s="21"/>
@@ -2253,10 +2273,10 @@
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="21"/>
       <c r="B16" s="22" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C16" s="20" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D16" s="21"/>
       <c r="E16" s="21"/>
@@ -2323,10 +2343,10 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="C29" s="10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D29" s="11">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated Attack Surface Analysis - Model Creation procedure / template (match threat model creation process type / class information) / fixed bad file location
</commit_message>
<xml_diff>
--- a/distribution/reference_documents/templates/AVCDL attack surface analysis model template.xlsx
+++ b/distribution/reference_documents/templates/AVCDL attack surface analysis model template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charles.wilson/Documents/projects/AVCDL/source/reference_documents/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16BFF26B-DA7D-0B4A-B05A-B9D102082DDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11610AF6-4B12-3E44-95EC-2BA399965B57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="41840" yWindow="940" windowWidth="30240" windowHeight="18880" xr2:uid="{DEA20EDE-F7A8-FC4F-9F8A-95A2B1030BD3}"/>
+    <workbookView xWindow="42140" yWindow="15320" windowWidth="30240" windowHeight="18880" activeTab="7" xr2:uid="{DEA20EDE-F7A8-FC4F-9F8A-95A2B1030BD3}"/>
   </bookViews>
   <sheets>
     <sheet name="cover sheet" sheetId="7" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="98">
   <si>
     <t>DO NOT EDIT THIS PAGE</t>
   </si>
@@ -192,19 +192,7 @@
     <t>process type</t>
   </si>
   <si>
-    <t>kernel</t>
-  </si>
-  <si>
-    <t>system</t>
-  </si>
-  <si>
     <t>service/daemon</t>
-  </si>
-  <si>
-    <t>user</t>
-  </si>
-  <si>
-    <t>process owner</t>
   </si>
   <si>
     <t>Element Name</t>
@@ -351,6 +339,24 @@
   <si>
     <t>other</t>
   </si>
+  <si>
+    <t>driver</t>
+  </si>
+  <si>
+    <t>process class</t>
+  </si>
+  <si>
+    <t>OS</t>
+  </si>
+  <si>
+    <t>third-party</t>
+  </si>
+  <si>
+    <t>self</t>
+  </si>
+  <si>
+    <t>external</t>
+  </si>
 </sst>
 </file>
 
@@ -359,7 +365,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yyyy;@"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -450,6 +456,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -511,7 +530,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -574,6 +593,11 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -918,7 +942,7 @@
   <sheetData>
     <row r="2" spans="2:11" ht="63" x14ac:dyDescent="0.75">
       <c r="B2" s="24" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C2" s="24"/>
       <c r="D2" s="24"/>
@@ -932,11 +956,11 @@
     </row>
     <row r="4" spans="2:11" ht="32" x14ac:dyDescent="0.4">
       <c r="B4" s="8" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C4" s="6"/>
       <c r="D4" s="26" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E4" s="26"/>
       <c r="F4" s="26"/>
@@ -947,11 +971,11 @@
     </row>
     <row r="6" spans="2:11" ht="32" x14ac:dyDescent="0.4">
       <c r="B6" s="8" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C6" s="6"/>
       <c r="D6" s="26" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="E6" s="26"/>
       <c r="F6" s="26"/>
@@ -962,7 +986,7 @@
     </row>
     <row r="8" spans="2:11" ht="32" x14ac:dyDescent="0.4">
       <c r="B8" s="8" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C8" s="6"/>
       <c r="D8" s="26"/>
@@ -975,11 +999,11 @@
     </row>
     <row r="10" spans="2:11" ht="32" x14ac:dyDescent="0.4">
       <c r="B10" s="8" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="27" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E10" s="27"/>
       <c r="F10" s="27"/>
@@ -990,11 +1014,11 @@
     </row>
     <row r="12" spans="2:11" ht="32" x14ac:dyDescent="0.4">
       <c r="B12" s="8" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="27" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="E12" s="27"/>
       <c r="F12" s="27"/>
@@ -1005,11 +1029,11 @@
     </row>
     <row r="14" spans="2:11" ht="32" x14ac:dyDescent="0.4">
       <c r="B14" s="8" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="27" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E14" s="27"/>
       <c r="F14" s="27"/>
@@ -1020,7 +1044,7 @@
     </row>
     <row r="16" spans="2:11" ht="32" x14ac:dyDescent="0.4">
       <c r="B16" s="8" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C16" s="6"/>
       <c r="D16" s="28">
@@ -1035,7 +1059,7 @@
     </row>
     <row r="18" spans="2:11" ht="32" x14ac:dyDescent="0.4">
       <c r="B18" s="8" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="9">
@@ -1049,7 +1073,7 @@
     </row>
     <row r="20" spans="2:11" ht="32" x14ac:dyDescent="0.4">
       <c r="B20" s="25" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C20" s="25"/>
       <c r="D20" s="25"/>
@@ -1105,7 +1129,7 @@
   <sheetData>
     <row r="2" spans="1:7" ht="63" x14ac:dyDescent="0.75">
       <c r="B2" s="29" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -1116,13 +1140,13 @@
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
       <c r="B4" s="12" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -1131,7 +1155,7 @@
       </c>
       <c r="C5" s="17"/>
       <c r="D5" s="19" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -1228,7 +1252,7 @@
   <sheetData>
     <row r="2" spans="1:7" ht="63" x14ac:dyDescent="0.75">
       <c r="B2" s="29" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -1239,13 +1263,13 @@
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
       <c r="B4" s="14" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C4" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>68</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -1343,7 +1367,7 @@
   <sheetData>
     <row r="2" spans="2:10" ht="63" x14ac:dyDescent="0.75">
       <c r="B2" s="29" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -1356,7 +1380,7 @@
     </row>
     <row r="5" spans="2:10" ht="27" x14ac:dyDescent="0.35">
       <c r="B5" s="30" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C5" s="30"/>
       <c r="D5" s="30"/>
@@ -1392,7 +1416,7 @@
   <sheetData>
     <row r="2" spans="1:12" ht="63" x14ac:dyDescent="0.75">
       <c r="B2" s="29" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -1423,10 +1447,10 @@
         <v>4</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
@@ -1607,7 +1631,7 @@
   <sheetData>
     <row r="2" spans="1:12" ht="63" x14ac:dyDescent="0.75">
       <c r="B2" s="29" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -1637,10 +1661,10 @@
         <v>4</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
@@ -1824,7 +1848,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="23.1640625" customWidth="1"/>
     <col min="7" max="7" width="29.6640625" customWidth="1"/>
     <col min="8" max="8" width="13.5" bestFit="1" customWidth="1"/>
@@ -1833,7 +1857,7 @@
   <sheetData>
     <row r="2" spans="1:12" ht="63" x14ac:dyDescent="0.75">
       <c r="B2" s="29" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -1858,7 +1882,7 @@
         <v>48</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>53</v>
+        <v>93</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>3</v>
@@ -1867,10 +1891,10 @@
         <v>4</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
@@ -2040,12 +2064,18 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="1">
-        <x14:dataValidation type="list" showInputMessage="1" showErrorMessage="1" xr:uid="{6750C4BD-2F34-2E41-A9D9-05C056381136}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
+        <x14:dataValidation type="list" showInputMessage="1" showErrorMessage="1" xr:uid="{0A79DC97-FEAA-CF49-95D8-51871EB2DBE7}">
           <x14:formula1>
-            <xm:f>legend!$D$2:$D$5</xm:f>
+            <xm:f>legend!$D$2:$D$4</xm:f>
           </x14:formula1>
           <xm:sqref>D5:D20</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{EC843808-0177-7141-9523-49F44CBE16BC}">
+          <x14:formula1>
+            <xm:f>legend!$F$2:$F$5</xm:f>
+          </x14:formula1>
+          <xm:sqref>E5:E20</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2055,15 +2085,16 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34E47EDA-BFD6-E448-BD76-322D521CE805}">
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="8.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="39.1640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>41</v>
       </c>
@@ -2077,10 +2108,13 @@
         <v>48</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+        <v>81</v>
+      </c>
+      <c r="F1" s="31" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="21" t="s">
         <v>46</v>
       </c>
@@ -2091,13 +2125,16 @@
         <v>40</v>
       </c>
       <c r="D2" s="21" t="s">
-        <v>49</v>
+        <v>84</v>
       </c>
       <c r="E2" s="21" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+        <v>82</v>
+      </c>
+      <c r="F2" s="22" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="21" t="s">
         <v>44</v>
       </c>
@@ -2108,13 +2145,16 @@
         <v>5</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>51</v>
+        <v>92</v>
       </c>
       <c r="E3" s="21" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+        <v>83</v>
+      </c>
+      <c r="F3" s="22" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="21" t="s">
         <v>45</v>
       </c>
@@ -2125,13 +2165,16 @@
         <v>6</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+        <v>84</v>
+      </c>
+      <c r="F4" s="22" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="21" t="s">
         <v>42</v>
       </c>
@@ -2141,14 +2184,15 @@
       <c r="C5" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="21" t="s">
-        <v>52</v>
-      </c>
+      <c r="D5" s="21"/>
       <c r="E5" s="21"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F5" s="22" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="21" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B6" s="22" t="s">
         <v>9</v>
@@ -2158,21 +2202,23 @@
       </c>
       <c r="D6" s="21"/>
       <c r="E6" s="21"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F6" s="22"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="21" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="D7" s="21"/>
       <c r="E7" s="21"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F7" s="20"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="21" t="s">
         <v>43</v>
       </c>
@@ -2184,10 +2230,11 @@
       </c>
       <c r="D8" s="21"/>
       <c r="E8" s="21"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F8" s="22"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="21" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B9" s="22" t="s">
         <v>13</v>
@@ -2197,10 +2244,11 @@
       </c>
       <c r="D9" s="21"/>
       <c r="E9" s="21"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F9" s="22"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="21" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B10" s="22" t="s">
         <v>15</v>
@@ -2210,10 +2258,11 @@
       </c>
       <c r="D10" s="21"/>
       <c r="E10" s="21"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F10" s="22"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="21" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B11" s="22" t="s">
         <v>17</v>
@@ -2223,10 +2272,11 @@
       </c>
       <c r="D11" s="21"/>
       <c r="E11" s="21"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F11" s="22"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="21" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B12" s="22" t="s">
         <v>19</v>
@@ -2236,8 +2286,9 @@
       </c>
       <c r="D12" s="21"/>
       <c r="E12" s="21"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F12" s="22"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="21"/>
       <c r="B13" s="22" t="s">
         <v>21</v>
@@ -2247,8 +2298,9 @@
       </c>
       <c r="D13" s="21"/>
       <c r="E13" s="21"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F13" s="22"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="21"/>
       <c r="B14" s="22" t="s">
         <v>23</v>
@@ -2258,30 +2310,33 @@
       </c>
       <c r="D14" s="21"/>
       <c r="E14" s="21"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F14" s="22"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="21"/>
       <c r="B15" s="22" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C15" s="20" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="D15" s="21"/>
       <c r="E15" s="21"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F15" s="20"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="21"/>
       <c r="B16" s="22" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C16" s="20" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D16" s="21"/>
       <c r="E16" s="21"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F16" s="20"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="21"/>
       <c r="B17" s="22" t="s">
         <v>25</v>
@@ -2291,8 +2346,9 @@
       </c>
       <c r="D17" s="21"/>
       <c r="E17" s="21"/>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F17" s="22"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="21"/>
       <c r="B18" s="22" t="s">
         <v>27</v>
@@ -2302,8 +2358,9 @@
       </c>
       <c r="D18" s="21"/>
       <c r="E18" s="21"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F18" s="22"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="21"/>
       <c r="B19" s="22" t="s">
         <v>29</v>
@@ -2313,8 +2370,9 @@
       </c>
       <c r="D19" s="21"/>
       <c r="E19" s="21"/>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F19" s="22"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="21"/>
       <c r="B20" s="22" t="s">
         <v>31</v>
@@ -2324,8 +2382,9 @@
       </c>
       <c r="D20" s="21"/>
       <c r="E20" s="21"/>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F20" s="22"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="21"/>
       <c r="B21" s="20" t="s">
         <v>33</v>
@@ -2335,19 +2394,31 @@
       </c>
       <c r="D21" s="21"/>
       <c r="E21" s="21"/>
-    </row>
-    <row r="25" spans="1:5" ht="380" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F21" s="20"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F22" s="32"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F23" s="32"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F24" s="32"/>
+    </row>
+    <row r="25" spans="1:6" ht="380" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="23" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F25" s="32"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="C29" s="10" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D29" s="11">
-        <v>4</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="F29" s="33"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:C21">

</xml_diff>